<commit_message>
Legent Member removide to accomodate long member name.
</commit_message>
<xml_diff>
--- a/members.xlsx
+++ b/members.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="60">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Hithesh Gowda </t>
   </si>
   <si>
-    <t xml:space="preserve">Subramanyam Umamaheshwaran </t>
+    <t xml:space="preserve">Subramanyam Umamaheshwaran</t>
   </si>
   <si>
     <t xml:space="preserve">Poornima Chittor Kashivishwanath </t>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t xml:space="preserve">Charish A jain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Individual </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sriharish Malebenur</t>
   </si>
 </sst>
 </file>
@@ -204,7 +210,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -233,12 +239,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -308,10 +308,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -320,12 +316,16 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -566,11 +566,11 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.16"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="4" style="1" width="22.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="8" style="1" width="18.88"/>
@@ -584,7 +584,7 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -602,550 +602,566 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="5" t="s">
+      <c r="A2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="4" t="n">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I3" s="4" t="n">
+      <c r="H3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="4" t="n">
+      <c r="H4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="4" t="n">
+      <c r="H5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="4" t="n">
+      <c r="H6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="4" t="n">
+      <c r="H7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" s="4" t="n">
+      <c r="H8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" s="4" t="n">
+      <c r="H9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I10" s="4" t="n">
+      <c r="H10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I11" s="4" t="n">
+      <c r="H11" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.5" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I12" s="4" t="n">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" s="4" t="n">
+      <c r="H13" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I14" s="4" t="n">
+      <c r="H14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I15" s="4" t="n">
+      <c r="H15" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" s="4" t="n">
+      <c r="H16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H17" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" s="4" t="n">
+      <c r="H17" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" s="4" t="n">
+      <c r="H18" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" s="4" t="n">
+      <c r="H19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" s="4" t="n">
+      <c r="H20" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" s="4" t="n">
+      <c r="H21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="G22" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H22" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" s="4" t="n">
+      <c r="H22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I22" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C23" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" s="4" t="n">
+      <c r="H23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I23" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="5" t="s">
+      <c r="A24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="5" t="n">
+      <c r="C24" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="G24" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I24" s="4" t="n">
+      <c r="H24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="5" t="s">
+      <c r="A25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H25" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" s="4" t="n">
+      <c r="H25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I25" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="5" t="s">
+      <c r="A26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I26" s="4" t="n">
+      <c r="H26" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="5" t="s">
+      <c r="A27" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C27" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" s="4" t="n">
+      <c r="H27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B28" s="5" t="s">
+      <c r="A28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" s="4" t="n">
+      <c r="H28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" s="3" t="n">
         <v>46387</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B29" s="5" t="s">
+      <c r="A29" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="G29" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H29" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>46387</v>
-      </c>
-    </row>
+      <c r="H29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>